<commit_message>
prepara deploy streamlit cloud
</commit_message>
<xml_diff>
--- a/reports/relatorio_2026_04.xlsx
+++ b/reports/relatorio_2026_04.xlsx
@@ -417,15 +417,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -457,6 +457,70 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>arquivo pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Claro</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>R$ 225,32</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>extraido</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sua Fatura Digital Claro chegou</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>downloads\pdfs\2026\Fatura Claro.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Claro</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>R$ 49,90</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>extraido</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sua Fatura Digital Claro chegou</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>downloads\pdfs\2026\SuaContaClaro_Abr-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>